<commit_message>
fix newton's method plot
</commit_message>
<xml_diff>
--- a/Plots/Comparison Table of k and p Values.xlsx
+++ b/Plots/Comparison Table of k and p Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/Assignment-1/Plots/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="8_{F5548F79-425C-4B76-B71C-57BD59B12E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54E985CD-A3E6-4B31-B6C0-858FC20D056F}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{F5548F79-425C-4B76-B71C-57BD59B12E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2F6BD4C-BBEF-4D68-A110-3A497DD32E91}"/>
   <bookViews>
     <workbookView xWindow="3000" yWindow="3000" windowWidth="17280" windowHeight="8880" xr2:uid="{D244108E-BDF8-4038-A556-2A9E06F46F59}"/>
   </bookViews>
@@ -525,7 +525,7 @@
     <col min="1" max="1" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
     <col min="5" max="5" width="17.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>